<commit_message>
Version 4: soporte CSV, negocio y metadatos
</commit_message>
<xml_diff>
--- a/data/ventas_cliente.xlsx
+++ b/data/ventas_cliente.xlsx
@@ -419,17 +419,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>producto</t>
+          <t>Producto</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>cantidad</t>
+          <t>Cantidad</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>precio_unitario</t>
+          <t>Precio Unitario</t>
         </is>
       </c>
     </row>

</xml_diff>